<commit_message>
Update Concepts and Employee_Table Excel files with new data
</commit_message>
<xml_diff>
--- a/Concepts/Concepts.xlsx
+++ b/Concepts/Concepts.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHWAS SHARMA\Documents\Xcel_portfolio\Concepts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829B67DF-8262-4704-8ECB-D637F611BE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78A0B67-BF9E-4B1A-A46F-EB114E50179F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="3" activeTab="6" xr2:uid="{5494DA74-FC50-4B2E-97A8-E9863E62A463}"/>
+    <workbookView xWindow="0" yWindow="10" windowWidth="19420" windowHeight="11020" xr2:uid="{5494DA74-FC50-4B2E-97A8-E9863E62A463}"/>
   </bookViews>
   <sheets>
-    <sheet name="Basic functions" sheetId="7" r:id="rId1"/>
-    <sheet name="Filter" sheetId="3" r:id="rId2"/>
-    <sheet name="Filter (2)" sheetId="6" r:id="rId3"/>
-    <sheet name="index" sheetId="5" r:id="rId4"/>
-    <sheet name="Filter with multiple condition" sheetId="4" r:id="rId5"/>
-    <sheet name="approximate_match" sheetId="2" r:id="rId6"/>
-    <sheet name="conditions" sheetId="8" r:id="rId7"/>
+    <sheet name="if and ifs" sheetId="12" r:id="rId1"/>
+    <sheet name="mix_question" sheetId="11" r:id="rId2"/>
+    <sheet name="count_fuction" sheetId="10" r:id="rId3"/>
+    <sheet name="sumif and sumifs" sheetId="9" r:id="rId4"/>
+    <sheet name="Basic functions" sheetId="7" r:id="rId5"/>
+    <sheet name="Filter" sheetId="3" r:id="rId6"/>
+    <sheet name="Filter (2)" sheetId="6" r:id="rId7"/>
+    <sheet name="index" sheetId="5" r:id="rId8"/>
+    <sheet name="Filter with multiple condition" sheetId="4" r:id="rId9"/>
+    <sheet name="approximate_match" sheetId="2" r:id="rId10"/>
+    <sheet name="conditions" sheetId="8" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -62,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="243">
   <si>
     <t>Jan</t>
   </si>
@@ -497,6 +501,300 @@
   </si>
   <si>
     <t>Costumer Name</t>
+  </si>
+  <si>
+    <t>Q: Total Sales of Burgur orders with Qty &gt; 10 (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Q: Total Sales in the East region where Sales &gt; 4000 (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Q: Total Qty sold where Sales &gt; 5000 (SUMIF).</t>
+  </si>
+  <si>
+    <t>Q: Total Sales of Pizza sold in the East region (SUMIFS).</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Burgur</t>
+  </si>
+  <si>
+    <t>Q: Total Sales of Burgur sold in the West region (SUMIFS).</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>Pizza</t>
+  </si>
+  <si>
+    <t>Q: Total Sales where Sales &gt; 5000 (SUMIF).</t>
+  </si>
+  <si>
+    <t>Pasta</t>
+  </si>
+  <si>
+    <t>Q: Total Qty sold of Pizza (SUMIF).</t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>Q: Total Sales in the East region (SUMIF).</t>
+  </si>
+  <si>
+    <t>Q: Total Sales of Burgur (SUMIF).</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Q: Average Salary of Male employees (AVERAGEIF).</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Q: Total Salary of employees whose name starts with 'M' (SUMIF, wildcard).</t>
+  </si>
+  <si>
+    <t>Sneha</t>
+  </si>
+  <si>
+    <t>Q: Total Salary of HR + IT departments combined (two SUMIFs added).</t>
+  </si>
+  <si>
+    <t>Q: Total Salary of all employees earning more than 35000 (SUMIF).</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Mohan</t>
+  </si>
+  <si>
+    <t>Q: Total Salary of Finance dept, Female employees (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Maya</t>
+  </si>
+  <si>
+    <t>Q: Total Salary of the HR department (SUMIF).</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Q: Count North + Product='B' orders with Sales &gt; 6000 (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Q: Count blank Price cells (COUNTBLANK).</t>
+  </si>
+  <si>
+    <t>Q: Count South orders with Sales &lt; 4000 (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Q: Count all non-empty Qty entries, incl. text (COUNTA).</t>
+  </si>
+  <si>
+    <t>Q: Count Product='A' orders with Sales &gt;= 5000 (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Q: Count numeric Qty entries (COUNT).</t>
+  </si>
+  <si>
+    <t>Q: Count orders with Sales &gt; 4000 (COUNTIF).</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>xyz</t>
+  </si>
+  <si>
+    <t>Q: Count Region='North' AND Product='A' orders (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Q: Count students scoring between 50 and 90 inclusive (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Aditi</t>
+  </si>
+  <si>
+    <t>Q: Count Male employees in IT dept (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Q: Count students scoring below 50 (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count how many attendance entries are filled in (COUNTA).</t>
+  </si>
+  <si>
+    <t>Absent</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>Q: Count Female employees (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count Rohan's Maths entries scoring above 90 (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Rohan</t>
+  </si>
+  <si>
+    <t>Q: Count names starting with 'R' (COUNTIF, wildcard).</t>
+  </si>
+  <si>
+    <t>Present</t>
+  </si>
+  <si>
+    <t>Ritu</t>
+  </si>
+  <si>
+    <t>Q: Count all non-empty cells in A1:D7 (COUNTA).</t>
+  </si>
+  <si>
+    <t>Q: Count Neha's entries scoring above 60 (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Q: Count employees whose Status = Absent (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count numeric cells in A1:D7 (COUNT).</t>
+  </si>
+  <si>
+    <t>Q: Count how many Maths entries there are (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count how many times "Ravi" appears (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count students scoring above 80 (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Q: Count employees whose Status = Present (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>EmpID</t>
+  </si>
+  <si>
+    <t>Find how many employees are in Pooja's Department AND Pooja's City (COUNTIFS, full sheet reference).</t>
+  </si>
+  <si>
+    <t>Find total Salary of Present, Sales-dept employees in Amit's City (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Find how many employees are in Ravi's Department AND Amit's City (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Find total Salary of Present employees in Pooja's Department (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Find total Bonus of Present employees in Pooja's City (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Find total Salary of employees in Neha's City AND Amit's Department (SUMIFS).</t>
+  </si>
+  <si>
+    <t>Find total Salary of employees with Amit's Status (SUMIF).</t>
+  </si>
+  <si>
+    <t>Simran</t>
+  </si>
+  <si>
+    <t>Find total Salary of employees in Amit's Department (SUMIF).</t>
+  </si>
+  <si>
+    <t>Find how many employees share Amit's City AND Status (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Find how many employees share Amit's Status AND Department (COUNTIFS).</t>
+  </si>
+  <si>
+    <t>Find how many employees are in the same Department as Amit (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Find how many employees have the same Status as Amit (COUNTIF).</t>
+  </si>
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Salary&gt;20000?</t>
+  </si>
+  <si>
+    <t>Bonus</t>
+  </si>
+  <si>
+    <t>Bonus Eligibility (IF, Sales&gt;=5000)</t>
+  </si>
+  <si>
+    <t>Salary Band (IFS)</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Nikita</t>
+  </si>
+  <si>
+    <t>Divyansh</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Uma</t>
+  </si>
+  <si>
+    <t>vedik</t>
+  </si>
+  <si>
+    <t>Vishwas</t>
+  </si>
+  <si>
+    <t>Pass/Fail (IF/AND, Marks&gt;=50 and Attendance&gt;=75)</t>
+  </si>
+  <si>
+    <t>Attendence</t>
+  </si>
+  <si>
+    <t>Pass/Fail (IF/OR, Marks&gt;=50 or Sports)</t>
+  </si>
+  <si>
+    <t>Sports</t>
+  </si>
+  <si>
+    <t>Pass/Fail (IF, Marks&gt;=50)</t>
   </si>
 </sst>
 </file>
@@ -586,7 +884,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -647,8 +945,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79989013336588644"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79989013336588644"/>
+        <bgColor rgb="FFDEEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFE2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFDEEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="30">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -985,13 +1307,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
@@ -1080,15 +1439,73 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="10" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1404,6 +1821,2097 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FAA2D9F-3756-4009-8C31-CF57B88A78F1}">
+  <dimension ref="A1:R16"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="7" width="8.6328125" style="1"/>
+    <col min="8" max="10" width="8" style="1" customWidth="1"/>
+    <col min="11" max="11" width="32" style="1" customWidth="1"/>
+    <col min="12" max="14" width="8.6328125" style="1"/>
+    <col min="15" max="16" width="8" style="1" customWidth="1"/>
+    <col min="17" max="17" width="12" style="1" customWidth="1"/>
+    <col min="18" max="18" width="38" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.6328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="R1" s="9" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="4">
+        <v>85</v>
+      </c>
+      <c r="C2" s="4" t="str">
+        <f>IF(B2&gt;=50,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4">
+        <v>30</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="K2" s="4" t="str">
+        <f>IF(OR(I2&gt;=50,J2="Yes"),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" s="4">
+        <v>80</v>
+      </c>
+      <c r="Q2" s="4">
+        <v>90</v>
+      </c>
+      <c r="R2" s="4" t="str">
+        <f>IF(AND(P2&gt;=50,Q2&gt;=75),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B3" s="4">
+        <v>45</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <f>IF(B3&gt;=50,"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="4">
+        <v>60</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K3" s="4" t="str">
+        <f>IF(OR(I3&gt;=50,J3="Yes"),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="P3" s="4">
+        <v>40</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>95</v>
+      </c>
+      <c r="R3" s="4" t="str">
+        <f>IF(AND(P3&gt;=50,Q3&gt;=75),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B4" s="4">
+        <v>60</v>
+      </c>
+      <c r="C4" s="4" t="str">
+        <f>IF(B4&gt;=50,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4">
+        <v>40</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="K4" s="4" t="str">
+        <f>IF(OR(I4&gt;=50,J4="Yes"),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="P4" s="4">
+        <v>70</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>60</v>
+      </c>
+      <c r="R4" s="4" t="str">
+        <f>IF(AND(P4&gt;=50,Q4&gt;=75),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="4">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <f>IF(B5&gt;=50,"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="4">
+        <v>80</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K5" s="4" t="str">
+        <f>IF(OR(I5&gt;=50,J5="Yes"),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="P5" s="4">
+        <v>55</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>85</v>
+      </c>
+      <c r="R5" s="4" t="str">
+        <f>IF(AND(P5&gt;=50,Q5&gt;=75),"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="4">
+        <v>75</v>
+      </c>
+      <c r="C6" s="4" t="str">
+        <f>IF(B6&gt;=50,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I6" s="4">
+        <v>20</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K6" s="4" t="str">
+        <f>IF(OR(I6&gt;=50,J6="Yes"),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="P6" s="4">
+        <v>30</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>50</v>
+      </c>
+      <c r="R6" s="4" t="str">
+        <f>IF(AND(P6&gt;=50,Q6&gt;=75),"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="68.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="73">
+        <v>10000</v>
+      </c>
+      <c r="C12" s="4" t="str">
+        <f t="array" ref="C12">_xlfn.IFS(B12&gt;=30000,"High",B12&gt;=20000,"Medium",B12&lt;20000,"Low")</f>
+        <v>Low</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" s="73">
+        <v>5000</v>
+      </c>
+      <c r="J12" s="4" t="str">
+        <f>IF(I12&gt;=5000,"Bonus","No Bonus")</f>
+        <v>Bonus</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="73">
+        <v>25000</v>
+      </c>
+      <c r="C13" s="4" t="str">
+        <f t="array" ref="C13">_xlfn.IFS(B13&gt;=30000,"High",B13&gt;=20000,"Medium",B13&lt;20000,"Low")</f>
+        <v>Medium</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" s="73">
+        <v>2000</v>
+      </c>
+      <c r="J13" s="4" t="str">
+        <f>IF(I13&gt;=5000,"Bonus","No Bonus")</f>
+        <v>No Bonus</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="73">
+        <v>40000</v>
+      </c>
+      <c r="C14" s="4" t="str">
+        <f t="array" ref="C14">_xlfn.IFS(B14&gt;=30000,"High",B14&gt;=20000,"Medium",B14&lt;20000,"Low")</f>
+        <v>High</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="73">
+        <v>8000</v>
+      </c>
+      <c r="J14" s="4" t="str">
+        <f>IF(I14&gt;=5000,"Bonus","No Bonus")</f>
+        <v>Bonus</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="73">
+        <v>15000</v>
+      </c>
+      <c r="C15" s="4" t="str">
+        <f t="array" ref="C15">_xlfn.IFS(B15&gt;=30000,"High",B15&gt;=20000,"Medium",B15&lt;20000,"Low")</f>
+        <v>Low</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="73">
+        <v>1500</v>
+      </c>
+      <c r="J15" s="4" t="str">
+        <f>IF(I15&gt;=5000,"Bonus","No Bonus")</f>
+        <v>No Bonus</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" s="73">
+        <v>30000</v>
+      </c>
+      <c r="C16" s="4" t="str">
+        <f t="array" ref="C16">_xlfn.IFS(B16&gt;=30000,"High",B16&gt;=20000,"Medium",B16&lt;20000,"Low")</f>
+        <v>High</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I16" s="73">
+        <v>6000</v>
+      </c>
+      <c r="J16" s="4" t="str">
+        <f>IF(I16&gt;=5000,"Bonus","No Bonus")</f>
+        <v>Bonus</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6330FB64-B819-4F03-968A-364C730BC8CC}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="3" max="3" width="70.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" style="1"/>
+    <col min="6" max="6" width="68.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.6328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="7" t="str">
+        <f>VLOOKUP(D2,A1:B6,2,1)</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="10">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>40</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>60</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>75</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>90</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="68.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4">
+        <v>110</v>
+      </c>
+      <c r="C11" s="4">
+        <v>105</v>
+      </c>
+      <c r="D11" s="4">
+        <v>106</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="7">
+        <f>VLOOKUP(F12,A10:D13,MATCH(F13,A10:D10,0),0)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4">
+        <v>110</v>
+      </c>
+      <c r="C12" s="4">
+        <v>104</v>
+      </c>
+      <c r="D12" s="4">
+        <v>105</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4">
+        <v>103</v>
+      </c>
+      <c r="C13" s="4">
+        <v>100</v>
+      </c>
+      <c r="D13" s="4">
+        <v>106</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B11E857-C61C-4876-8EC4-54E8C7146BF1}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.453125" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" customWidth="1"/>
+    <col min="3" max="3" width="24.6328125" customWidth="1"/>
+    <col min="4" max="4" width="8.6328125" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="13.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="68" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="68" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="68" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" s="68" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="69" t="s">
+        <v>140</v>
+      </c>
+      <c r="G1" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="67" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="66" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="65">
+        <v>11668</v>
+      </c>
+      <c r="C2" s="65">
+        <v>6</v>
+      </c>
+      <c r="D2" s="65" t="str">
+        <f t="shared" ref="D2:D10" si="0">IF(B2&gt;5000,"10%","0")</f>
+        <v>10%</v>
+      </c>
+      <c r="E2" s="65" t="str">
+        <f>IF(OR(B2&gt;10000,C2&gt;4),"20%","0")</f>
+        <v>20%</v>
+      </c>
+      <c r="F2" s="65" t="str">
+        <f t="shared" ref="F2:F10" si="1">IF(AND(B2&gt;20000,C2&gt;9),"30%","0")</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="65" t="str" cm="1">
+        <f t="array" ref="G2">_xlfn.IFS(B2&gt;20000,"A",B2&gt;10000,"B",B2&lt;10000,"C")</f>
+        <v>B</v>
+      </c>
+      <c r="H2" s="65" t="str">
+        <f t="shared" ref="H2:H10" si="2">IF(B2&gt;20000,"A",IF(B2&gt;10000,"B",IF(B2&lt;10000,"C")))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="66" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="65">
+        <v>43316</v>
+      </c>
+      <c r="C3" s="65">
+        <v>6</v>
+      </c>
+      <c r="D3" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E3" s="65" t="str">
+        <f t="shared" ref="E3:E10" si="3">IF(OR(B3&gt;10000,C3&gt;4),"20%")</f>
+        <v>20%</v>
+      </c>
+      <c r="F3" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G3" s="65" t="str" cm="1">
+        <f t="array" ref="G3">_xlfn.IFS(B3&gt;20000,"A",B3&gt;10000,"B",B3&lt;10000,"C")</f>
+        <v>A</v>
+      </c>
+      <c r="H3" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="66" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="65">
+        <v>13951</v>
+      </c>
+      <c r="C4" s="65">
+        <v>4</v>
+      </c>
+      <c r="D4" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E4" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F4" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="65" t="str" cm="1">
+        <f t="array" ref="G4">_xlfn.IFS(B4&gt;20000,"A",B4&gt;10000,"B",B4&lt;10000,"C")</f>
+        <v>B</v>
+      </c>
+      <c r="H4" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5" s="65">
+        <v>10488</v>
+      </c>
+      <c r="C5" s="65">
+        <v>14</v>
+      </c>
+      <c r="D5" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E5" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F5" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="65" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.IFS(B5&gt;20000,"A",B5&gt;10000,"B",B5&lt;10000,"C")</f>
+        <v>B</v>
+      </c>
+      <c r="H5" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="66" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="65">
+        <v>33641</v>
+      </c>
+      <c r="C6" s="65">
+        <v>10</v>
+      </c>
+      <c r="D6" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E6" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F6" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>30%</v>
+      </c>
+      <c r="G6" s="65" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.IFS(B6&gt;20000,"A",B6&gt;10000,"B",B6&lt;10000,"C")</f>
+        <v>A</v>
+      </c>
+      <c r="H6" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="66" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="65">
+        <v>26146</v>
+      </c>
+      <c r="C7" s="65">
+        <v>15</v>
+      </c>
+      <c r="D7" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E7" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F7" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>30%</v>
+      </c>
+      <c r="G7" s="65" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.IFS(B7&gt;20000,"A",B7&gt;10000,"B",B7&lt;10000,"C")</f>
+        <v>A</v>
+      </c>
+      <c r="H7" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="66" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="65">
+        <v>30080</v>
+      </c>
+      <c r="C8" s="65">
+        <v>4</v>
+      </c>
+      <c r="D8" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E8" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F8" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="65" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.IFS(B8&gt;20000,"A",B8&gt;10000,"B",B8&lt;10000,"C")</f>
+        <v>A</v>
+      </c>
+      <c r="H8" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="66" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="65">
+        <v>32446</v>
+      </c>
+      <c r="C9" s="65">
+        <v>13</v>
+      </c>
+      <c r="D9" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E9" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F9" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>30%</v>
+      </c>
+      <c r="G9" s="65" t="str" cm="1">
+        <f t="array" ref="G9">_xlfn.IFS(B9&gt;20000,"A",B9&gt;10000,"B",B9&lt;10000,"C")</f>
+        <v>A</v>
+      </c>
+      <c r="H9" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="66" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" s="65">
+        <v>13153</v>
+      </c>
+      <c r="C10" s="65">
+        <v>8</v>
+      </c>
+      <c r="D10" s="65" t="str">
+        <f t="shared" si="0"/>
+        <v>10%</v>
+      </c>
+      <c r="E10" s="65" t="str">
+        <f t="shared" si="3"/>
+        <v>20%</v>
+      </c>
+      <c r="F10" s="65" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="65" t="str" cm="1">
+        <f t="array" ref="G10">_xlfn.IFS(B10&gt;20000,"A",B10&gt;10000,"B",B10&lt;10000,"C")</f>
+        <v>B</v>
+      </c>
+      <c r="H10" s="65" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="64"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="64"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{697DEFB5-3E64-4D31-A8CA-DC3BE6E47861}">
+  <dimension ref="A2:L14"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10" style="1" customWidth="1"/>
+    <col min="7" max="8" width="12" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6328125" style="1"/>
+    <col min="11" max="12" width="24" style="1" customWidth="1"/>
+    <col min="13" max="21" width="1.81640625" style="1" customWidth="1"/>
+    <col min="22" max="43" width="2.81640625" style="1" customWidth="1"/>
+    <col min="44" max="16384" width="8.6328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="96" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="96" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="96" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" s="96" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="96" t="s">
+        <v>227</v>
+      </c>
+      <c r="F2" s="96" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="95" t="s">
+        <v>226</v>
+      </c>
+      <c r="I2" s="94" t="s">
+        <v>83</v>
+      </c>
+      <c r="K2" s="93" t="s">
+        <v>225</v>
+      </c>
+      <c r="L2" s="93"/>
+    </row>
+    <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="81" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D3" s="80">
+        <v>20000</v>
+      </c>
+      <c r="E3" s="80">
+        <v>2000</v>
+      </c>
+      <c r="F3" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="92" t="str">
+        <f>IF(D3&gt;20000,"True","False")</f>
+        <v>False</v>
+      </c>
+      <c r="I3" s="90">
+        <f>COUNTIF(C3:C9,C3)</f>
+        <v>5</v>
+      </c>
+      <c r="K3" s="89" t="s">
+        <v>224</v>
+      </c>
+      <c r="L3" s="89"/>
+    </row>
+    <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="D4" s="80">
+        <v>25000</v>
+      </c>
+      <c r="E4" s="80">
+        <v>3000</v>
+      </c>
+      <c r="F4" s="81" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="92" t="str">
+        <f>IF(D4&gt;20000,"True","False")</f>
+        <v>True</v>
+      </c>
+      <c r="I4" s="90">
+        <f>COUNTIF(B3:B9,B3)</f>
+        <v>3</v>
+      </c>
+      <c r="K4" s="89" t="s">
+        <v>223</v>
+      </c>
+      <c r="L4" s="89"/>
+    </row>
+    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="81" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" s="80">
+        <v>18000</v>
+      </c>
+      <c r="E5" s="80">
+        <v>1500</v>
+      </c>
+      <c r="F5" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="92" t="str">
+        <f>IF(D5&gt;20000,"True","False")</f>
+        <v>False</v>
+      </c>
+      <c r="I5" s="90">
+        <f>COUNTIFS(C3:C9,C3,B3:B9,B3)</f>
+        <v>2</v>
+      </c>
+      <c r="K5" s="89" t="s">
+        <v>222</v>
+      </c>
+      <c r="L5" s="89"/>
+    </row>
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="81" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D6" s="80">
+        <v>30000</v>
+      </c>
+      <c r="E6" s="80">
+        <v>4000</v>
+      </c>
+      <c r="F6" s="81" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="92" t="str">
+        <f>IF(D6&gt;20000,"True","False")</f>
+        <v>True</v>
+      </c>
+      <c r="I6" s="90">
+        <f>COUNTIFS(F3:F9,F3,C3:C9,C3)</f>
+        <v>3</v>
+      </c>
+      <c r="K6" s="89" t="s">
+        <v>221</v>
+      </c>
+      <c r="L6" s="89"/>
+    </row>
+    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="81" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D7" s="80">
+        <v>22000</v>
+      </c>
+      <c r="E7" s="80">
+        <v>2000</v>
+      </c>
+      <c r="F7" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="92" t="str">
+        <f>IF(D7&gt;20000,"True","False")</f>
+        <v>True</v>
+      </c>
+      <c r="I7" s="90">
+        <f>SUMIF(B3:B9,B3,D3:D9)</f>
+        <v>59000</v>
+      </c>
+      <c r="K7" s="89" t="s">
+        <v>220</v>
+      </c>
+      <c r="L7" s="89"/>
+    </row>
+    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="81" t="s">
+        <v>219</v>
+      </c>
+      <c r="B8" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="D8" s="80">
+        <v>21000</v>
+      </c>
+      <c r="E8" s="80">
+        <v>2500</v>
+      </c>
+      <c r="F8" s="81" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="92" t="str">
+        <f>IF(D8&gt;20000,"True","False")</f>
+        <v>True</v>
+      </c>
+      <c r="I8" s="90">
+        <f>SUMIF(C3:C9,C3,D3:D9)</f>
+        <v>118000</v>
+      </c>
+      <c r="K8" s="89" t="s">
+        <v>218</v>
+      </c>
+      <c r="L8" s="89"/>
+    </row>
+    <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="80">
+        <v>28000</v>
+      </c>
+      <c r="E9" s="80">
+        <v>3500</v>
+      </c>
+      <c r="F9" s="81" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="92" t="str">
+        <f>IF(D9&gt;20000,"True","False")</f>
+        <v>True</v>
+      </c>
+      <c r="I9" s="90">
+        <f>SUMIFS(D3:D9,F3:F9,F3,B3:B9,B4)</f>
+        <v>22000</v>
+      </c>
+      <c r="K9" s="89" t="s">
+        <v>217</v>
+      </c>
+      <c r="L9" s="89"/>
+    </row>
+    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G10" s="91"/>
+      <c r="I10" s="90">
+        <f>SUMIFS(E3:E9,C3:C9,C3,F3:F9,F6)</f>
+        <v>7500</v>
+      </c>
+      <c r="K10" s="89" t="s">
+        <v>216</v>
+      </c>
+      <c r="L10" s="89"/>
+    </row>
+    <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G11" s="91"/>
+      <c r="I11" s="90">
+        <f>SUMIFS(D3:D9,B3:B9,B6,C3:C9,C3)</f>
+        <v>58000</v>
+      </c>
+      <c r="K11" s="89" t="s">
+        <v>215</v>
+      </c>
+      <c r="L11" s="89"/>
+    </row>
+    <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G12" s="91"/>
+      <c r="I12" s="90">
+        <f>COUNTIFS(B3:B9,B5,F3:F9,F3)</f>
+        <v>2</v>
+      </c>
+      <c r="K12" s="89" t="s">
+        <v>214</v>
+      </c>
+      <c r="L12" s="89"/>
+    </row>
+    <row r="13" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G13" s="91"/>
+      <c r="I13" s="90">
+        <f>SUMIFS(D3:D9,C3:C9,C3,B3:B9,B3,F3:F9,F3)</f>
+        <v>38000</v>
+      </c>
+      <c r="K13" s="89" t="s">
+        <v>213</v>
+      </c>
+      <c r="L13" s="89"/>
+    </row>
+    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G14" s="91"/>
+      <c r="I14" s="90">
+        <f>COUNTIFS(mix_question!C3:C9,mix_question!C3,mix_question!B3:B9,mix_question!B6,mix_question!F3:F9,mix_question!F6)</f>
+        <v>2</v>
+      </c>
+      <c r="K14" s="89" t="s">
+        <v>212</v>
+      </c>
+      <c r="L14" s="89"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K12:L12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD81181-385F-4483-99AA-E82D715EEBD6}">
+  <dimension ref="A1:U21"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="3" max="4" width="8" style="1" customWidth="1"/>
+    <col min="5" max="5" width="41.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.6328125" style="1"/>
+    <col min="10" max="11" width="7" style="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="1" customWidth="1"/>
+    <col min="13" max="13" width="52.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="1.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7" style="1" customWidth="1"/>
+    <col min="16" max="17" width="8" style="1" customWidth="1"/>
+    <col min="18" max="18" width="7" style="1" customWidth="1"/>
+    <col min="19" max="19" width="8" style="1" customWidth="1"/>
+    <col min="20" max="20" width="47.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="1.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="8.6328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="83" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="83" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="83" t="s">
+        <v>173</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="83" t="s">
+        <v>211</v>
+      </c>
+      <c r="K1" s="83" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="88" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q1" s="83" t="s">
+        <v>209</v>
+      </c>
+      <c r="R1" s="83" t="s">
+        <v>208</v>
+      </c>
+      <c r="S1" s="83" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="81" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="81" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="85">
+        <v>30000</v>
+      </c>
+      <c r="J2" s="81">
+        <v>101</v>
+      </c>
+      <c r="K2" s="81" t="s">
+        <v>193</v>
+      </c>
+      <c r="L2" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="M2" s="87" t="s">
+        <v>207</v>
+      </c>
+      <c r="N2" s="79">
+        <f>COUNTIF(L2:L6,L4)</f>
+        <v>3</v>
+      </c>
+      <c r="Q2" s="81" t="s">
+        <v>188</v>
+      </c>
+      <c r="R2" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="S2" s="81">
+        <v>78</v>
+      </c>
+      <c r="T2" s="84" t="s">
+        <v>206</v>
+      </c>
+      <c r="U2" s="79">
+        <f>COUNTIF(S2:S7,"&gt;80")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="81" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="81" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="85">
+        <v>28000</v>
+      </c>
+      <c r="J3" s="81">
+        <v>102</v>
+      </c>
+      <c r="K3" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="M3" s="79" t="s">
+        <v>205</v>
+      </c>
+      <c r="N3" s="79">
+        <f>COUNTIF(K2:K6,K6)</f>
+        <v>2</v>
+      </c>
+      <c r="Q3" s="81" t="s">
+        <v>196</v>
+      </c>
+      <c r="R3" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="S3" s="81">
+        <v>90</v>
+      </c>
+      <c r="T3" s="84" t="s">
+        <v>204</v>
+      </c>
+      <c r="U3" s="79">
+        <f>COUNTIF(R2:R7,R2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="81" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="81" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="85">
+        <v>45000</v>
+      </c>
+      <c r="E4" s="79" t="s">
+        <v>203</v>
+      </c>
+      <c r="F4" s="79">
+        <f>COUNT(A1:D7)</f>
+        <v>6</v>
+      </c>
+      <c r="J4" s="81">
+        <v>103</v>
+      </c>
+      <c r="K4" s="81" t="s">
+        <v>80</v>
+      </c>
+      <c r="L4" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="M4" s="79" t="s">
+        <v>202</v>
+      </c>
+      <c r="N4" s="79">
+        <f>COUNTIF(L2:L6,L3)</f>
+        <v>2</v>
+      </c>
+      <c r="Q4" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="R4" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="S4" s="81">
+        <v>55</v>
+      </c>
+      <c r="T4" s="84" t="s">
+        <v>201</v>
+      </c>
+      <c r="U4" s="79">
+        <f>COUNTIFS(Q2:Q7,Q4,S2:S7,"&gt;60")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="81" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="81" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="81" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="85">
+        <v>35000</v>
+      </c>
+      <c r="E5" s="79" t="s">
+        <v>200</v>
+      </c>
+      <c r="F5" s="79">
+        <f>COUNTA(A1:D7)</f>
+        <v>28</v>
+      </c>
+      <c r="J5" s="81">
+        <v>104</v>
+      </c>
+      <c r="K5" s="81" t="s">
+        <v>199</v>
+      </c>
+      <c r="L5" s="81" t="s">
+        <v>198</v>
+      </c>
+      <c r="M5" s="86" t="s">
+        <v>197</v>
+      </c>
+      <c r="N5" s="79">
+        <f>COUNTIF(K2:K6,"R*")</f>
+        <v>3</v>
+      </c>
+      <c r="Q5" s="81" t="s">
+        <v>196</v>
+      </c>
+      <c r="R5" s="81" t="s">
+        <v>127</v>
+      </c>
+      <c r="S5" s="81">
+        <v>92</v>
+      </c>
+      <c r="T5" s="84" t="s">
+        <v>195</v>
+      </c>
+      <c r="U5" s="79">
+        <f>COUNTIFS(Q2:Q7,Q3,R2:R7,R2,S2:S7,"&gt;90")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="81" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="81" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" s="85">
+        <v>40000</v>
+      </c>
+      <c r="E6" s="79" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" s="79">
+        <f>COUNTIF(C2:C7,C5)</f>
+        <v>4</v>
+      </c>
+      <c r="J6" s="81">
+        <v>105</v>
+      </c>
+      <c r="K6" s="81" t="s">
+        <v>193</v>
+      </c>
+      <c r="L6" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="M6" s="86" t="s">
+        <v>191</v>
+      </c>
+      <c r="N6" s="79">
+        <f>COUNTA(L2:L6)</f>
+        <v>5</v>
+      </c>
+      <c r="Q6" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="R6" s="81" t="s">
+        <v>75</v>
+      </c>
+      <c r="S6" s="81">
+        <v>81</v>
+      </c>
+      <c r="T6" s="84" t="s">
+        <v>190</v>
+      </c>
+      <c r="U6" s="79">
+        <f>COUNTIF(S2:S7,"&lt;50")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="81" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="81" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" s="85">
+        <v>37000</v>
+      </c>
+      <c r="E7" s="79" t="s">
+        <v>189</v>
+      </c>
+      <c r="F7" s="79">
+        <f>COUNTIFS(C2:C7,C4,B2:B7,B3)</f>
+        <v>1</v>
+      </c>
+      <c r="Q7" s="81" t="s">
+        <v>188</v>
+      </c>
+      <c r="R7" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="S7" s="81">
+        <v>49</v>
+      </c>
+      <c r="T7" s="84" t="s">
+        <v>187</v>
+      </c>
+      <c r="U7" s="79">
+        <f>COUNTIFS(S2:S7,"&gt;=50",S2:S7,"&lt;=90")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="83" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="83" t="s">
+        <v>160</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="J15" s="83" t="s">
+        <v>161</v>
+      </c>
+      <c r="K15" s="83" t="s">
+        <v>7</v>
+      </c>
+      <c r="L15" s="83" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="81" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="81">
+        <v>10</v>
+      </c>
+      <c r="C16" s="79">
+        <v>200</v>
+      </c>
+      <c r="J16" s="81" t="s">
+        <v>176</v>
+      </c>
+      <c r="K16" s="81" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="80">
+        <v>5000</v>
+      </c>
+      <c r="M16" s="82" t="s">
+        <v>185</v>
+      </c>
+      <c r="N16" s="79">
+        <f>COUNTIF(J16:J21,J16)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="C17" s="79">
+        <v>150</v>
+      </c>
+      <c r="D17" s="79" t="s">
+        <v>183</v>
+      </c>
+      <c r="E17" s="79">
+        <f>COUNT(B16:B20)</f>
+        <v>4</v>
+      </c>
+      <c r="J17" s="81" t="s">
+        <v>149</v>
+      </c>
+      <c r="K17" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="L17" s="80">
+        <v>3000</v>
+      </c>
+      <c r="M17" s="82" t="s">
+        <v>182</v>
+      </c>
+      <c r="N17" s="79">
+        <f>COUNTIFS(J16:J21,J16,K16:K21,K16)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="81" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="81">
+        <v>25</v>
+      </c>
+      <c r="C18" s="79">
+        <v>300</v>
+      </c>
+      <c r="D18" s="79" t="s">
+        <v>181</v>
+      </c>
+      <c r="E18" s="79">
+        <f>COUNT(C16:C20)</f>
+        <v>4</v>
+      </c>
+      <c r="J18" s="81" t="s">
+        <v>176</v>
+      </c>
+      <c r="K18" s="81" t="s">
+        <v>8</v>
+      </c>
+      <c r="L18" s="80">
+        <v>6000</v>
+      </c>
+      <c r="M18" s="82" t="s">
+        <v>180</v>
+      </c>
+      <c r="N18" s="79">
+        <f>COUNTIF(L16:L21,"&gt;4000")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="81" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="81">
+        <v>0</v>
+      </c>
+      <c r="C19" s="79">
+        <v>400</v>
+      </c>
+      <c r="D19" s="79" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" s="79">
+        <f>COUNTA(B16:B20)</f>
+        <v>5</v>
+      </c>
+      <c r="J19" s="81" t="s">
+        <v>152</v>
+      </c>
+      <c r="K19" s="81" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="80">
+        <v>2000</v>
+      </c>
+      <c r="M19" s="82" t="s">
+        <v>178</v>
+      </c>
+      <c r="N19" s="79">
+        <f>COUNTIFS(K16:K21,K16,L16:L21,"&gt;=5000")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="81" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="81">
+        <v>15</v>
+      </c>
+      <c r="C20" s="79"/>
+      <c r="D20" s="79" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" s="79">
+        <f>COUNTBLANK(C16:C20)</f>
+        <v>1</v>
+      </c>
+      <c r="J20" s="81" t="s">
+        <v>176</v>
+      </c>
+      <c r="K20" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="L20" s="80">
+        <v>7000</v>
+      </c>
+      <c r="M20" s="82" t="s">
+        <v>175</v>
+      </c>
+      <c r="N20" s="79">
+        <f>COUNTIFS(J16:J21,J17,L16:L21,"&lt;4000")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J21" s="81" t="s">
+        <v>149</v>
+      </c>
+      <c r="K21" s="81" t="s">
+        <v>8</v>
+      </c>
+      <c r="L21" s="80">
+        <v>5000</v>
+      </c>
+      <c r="M21" s="79"/>
+      <c r="N21" s="79">
+        <f>COUNTIFS(J16:J21,J16,K16:K21,K17,L16:L21,"&gt;6000")</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCC3EEB-69DC-41D7-8498-8542E8631996}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" style="1"/>
+    <col min="6" max="6" width="46" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" style="1"/>
+    <col min="9" max="9" width="10" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.6328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="73">
+        <v>30000</v>
+      </c>
+      <c r="E2" s="78"/>
+      <c r="F2" s="77" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" s="76">
+        <f>SUMIF(B2:B7,B2,D2:D7)</f>
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="73">
+        <v>28000</v>
+      </c>
+      <c r="F3" s="77" t="s">
+        <v>170</v>
+      </c>
+      <c r="G3" s="76">
+        <f>SUMIFS(D2:D7,B2:B7,"Finance",C2:C7,"Female")</f>
+        <v>72000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="73">
+        <v>45000</v>
+      </c>
+      <c r="F4" s="77" t="s">
+        <v>167</v>
+      </c>
+      <c r="G4" s="76">
+        <f>SUMIF(D2:D7,"&gt;35000",D2:D7)</f>
+        <v>122000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="73">
+        <v>35000</v>
+      </c>
+      <c r="F5" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="G5" s="76">
+        <f>SUMIF(B2:B7,"HR",D2:D7)+SUMIF(B2:B7,"IT",D2:D7)</f>
+        <v>143000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" s="73">
+        <v>40000</v>
+      </c>
+      <c r="F6" s="77" t="s">
+        <v>164</v>
+      </c>
+      <c r="G6" s="76">
+        <f>SUMIF(A2:A7,"m*",D2:D7)</f>
+        <v>73000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" s="73">
+        <v>37000</v>
+      </c>
+      <c r="F7" s="75" t="s">
+        <v>162</v>
+      </c>
+      <c r="G7" s="74">
+        <f>AVERAGEIF(C2:C7,C4,D2:D7)</f>
+        <v>37500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="73">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="4">
+        <v>10</v>
+      </c>
+      <c r="F12" s="72" t="s">
+        <v>159</v>
+      </c>
+      <c r="G12" s="71">
+        <f>SUMIF(A12:A17,"Burgur",C12:C17)</f>
+        <v>16500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" s="73">
+        <v>7000</v>
+      </c>
+      <c r="D13" s="4">
+        <v>15</v>
+      </c>
+      <c r="F13" s="72" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" s="71">
+        <f>SUMIF(B12:B17,"East",C12:C17)</f>
+        <v>15500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="73">
+        <v>6000</v>
+      </c>
+      <c r="D14" s="4">
+        <v>12</v>
+      </c>
+      <c r="F14" s="72" t="s">
+        <v>156</v>
+      </c>
+      <c r="G14" s="71">
+        <f>SUMIF(A12:A17,"Pizza",D12:D17)</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C15" s="73">
+        <v>4000</v>
+      </c>
+      <c r="D15" s="4">
+        <v>8</v>
+      </c>
+      <c r="F15" s="72" t="s">
+        <v>154</v>
+      </c>
+      <c r="G15" s="71">
+        <f>SUMIF(C12:C17,"&gt;5000",C12:C17)</f>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="73">
+        <v>6500</v>
+      </c>
+      <c r="D16" s="4">
+        <v>14</v>
+      </c>
+      <c r="F16" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" s="71">
+        <f>SUMIFS(C12:C17,A12:A17,"Burgur",B12:B17,"West")</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C17" s="73">
+        <v>5500</v>
+      </c>
+      <c r="D17" s="4">
+        <v>11</v>
+      </c>
+      <c r="F17" s="72" t="s">
+        <v>148</v>
+      </c>
+      <c r="G17" s="71">
+        <f>SUMIFS(C12:C17,A12:A17,A13,B12:B17,B15)</f>
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F18" s="72" t="s">
+        <v>147</v>
+      </c>
+      <c r="G18" s="71">
+        <f>SUMIF(C12:C17,"&gt;5000",D12:D17)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F19" s="72" t="s">
+        <v>146</v>
+      </c>
+      <c r="G19" s="71">
+        <f>SUMIFS(C12:C17,B12:B17,B15,C12:C17,"&gt;4000")</f>
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F20" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="G20" s="71">
+        <f>SUMIFS(C12:C17,D12:D17,"&gt;10",A12:A17,A14)</f>
+        <v>11500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5EE1B86-25FA-4BB3-B26F-7F646CF8E109}">
   <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -1636,7 +4144,7 @@
       </c>
       <c r="D15" s="50">
         <f ca="1">TODAY()</f>
-        <v>46276</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -1645,7 +4153,7 @@
       </c>
       <c r="D16" s="53">
         <f ca="1">NOW()</f>
-        <v>46276.955199421296</v>
+        <v>46278.471532523145</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.25">
@@ -1690,7 +4198,7 @@
       </c>
       <c r="D21" s="50">
         <f ca="1">DATEDIF(D17,D15,"d")</f>
-        <v>7330</v>
+        <v>7332</v>
       </c>
     </row>
   </sheetData>
@@ -1698,7 +4206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D221076-561E-490B-B197-906FBF5C6BC9}">
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2030,7 +4538,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD67955-C821-4BC2-931F-07F693E43CEB}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2074,12 +4582,12 @@
       <c r="D2" s="17">
         <v>8</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="70" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
     </row>
     <row r="3" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="17">
@@ -2435,7 +4943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24E54DD6-712C-4076-81EE-50940DB44804}">
   <dimension ref="A1:M17"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2708,7 +5216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60478AA7-E19C-4A2B-93C4-F984A24E6CF2}">
   <dimension ref="A1:O26"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3221,489 +5729,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6330FB64-B819-4F03-968A-364C730BC8CC}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" width="70.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" style="1"/>
-    <col min="6" max="6" width="68.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.6328125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="7" t="str">
-        <f>VLOOKUP(D2,A1:B6,2,1)</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="4">
-        <v>0</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="10">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>40</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>60</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>75</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>90</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="68.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="10" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="4">
-        <v>110</v>
-      </c>
-      <c r="C11" s="4">
-        <v>105</v>
-      </c>
-      <c r="D11" s="4">
-        <v>106</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" s="7">
-        <f>VLOOKUP(F12,A10:D13,MATCH(F13,A10:D10,0),0)</f>
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="4">
-        <v>110</v>
-      </c>
-      <c r="C12" s="4">
-        <v>104</v>
-      </c>
-      <c r="D12" s="4">
-        <v>105</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="4">
-        <v>103</v>
-      </c>
-      <c r="C13" s="4">
-        <v>100</v>
-      </c>
-      <c r="D13" s="4">
-        <v>106</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B11E857-C61C-4876-8EC4-54E8C7146BF1}">
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="27.453125" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" customWidth="1"/>
-    <col min="3" max="3" width="24.6328125" customWidth="1"/>
-    <col min="4" max="4" width="8.6328125" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="13.90625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="69" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="69" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="69" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1" s="69" t="s">
-        <v>138</v>
-      </c>
-      <c r="E1" s="69" t="s">
-        <v>141</v>
-      </c>
-      <c r="F1" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="G1" s="69" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="68" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="67" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" s="66">
-        <v>11668</v>
-      </c>
-      <c r="C2" s="66">
-        <v>6</v>
-      </c>
-      <c r="D2" s="66" t="str">
-        <f>IF(B2&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E2" s="66" t="str">
-        <f>IF(OR(B2&gt;10000,C2&gt;4),"20%","0")</f>
-        <v>20%</v>
-      </c>
-      <c r="F2" s="66" t="str">
-        <f>IF(AND(B2&gt;20000,C2&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="66" t="str" cm="1">
-        <f t="array" ref="G2">_xlfn.IFS(B2&gt;20000,"A",B2&gt;10000,"B",B2&lt;10000,"C")</f>
-        <v>B</v>
-      </c>
-      <c r="H2" s="66" t="str">
-        <f>IF(B2&gt;20000,"A",IF(B2&gt;10000,"B",IF(B2&lt;10000,"C")))</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="67" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="66">
-        <v>43316</v>
-      </c>
-      <c r="C3" s="66">
-        <v>6</v>
-      </c>
-      <c r="D3" s="66" t="str">
-        <f>IF(B3&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E3" s="66" t="str">
-        <f>IF(OR(B3&gt;10000,C3&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F3" s="66" t="str">
-        <f>IF(AND(B3&gt;20000,C3&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="66" t="str" cm="1">
-        <f t="array" ref="G3">_xlfn.IFS(B3&gt;20000,"A",B3&gt;10000,"B",B3&lt;10000,"C")</f>
-        <v>A</v>
-      </c>
-      <c r="H3" s="66" t="str">
-        <f>IF(B3&gt;20000,"A",IF(B3&gt;10000,"B",IF(B3&lt;10000,"C")))</f>
-        <v>A</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="67" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="66">
-        <v>13951</v>
-      </c>
-      <c r="C4" s="66">
-        <v>4</v>
-      </c>
-      <c r="D4" s="66" t="str">
-        <f>IF(B4&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E4" s="66" t="str">
-        <f>IF(OR(B4&gt;10000,C4&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F4" s="66" t="str">
-        <f>IF(AND(B4&gt;20000,C4&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="66" t="str" cm="1">
-        <f t="array" ref="G4">_xlfn.IFS(B4&gt;20000,"A",B4&gt;10000,"B",B4&lt;10000,"C")</f>
-        <v>B</v>
-      </c>
-      <c r="H4" s="66" t="str">
-        <f>IF(B4&gt;20000,"A",IF(B4&gt;10000,"B",IF(B4&lt;10000,"C")))</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="67" t="s">
-        <v>134</v>
-      </c>
-      <c r="B5" s="66">
-        <v>10488</v>
-      </c>
-      <c r="C5" s="66">
-        <v>14</v>
-      </c>
-      <c r="D5" s="66" t="str">
-        <f>IF(B5&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E5" s="66" t="str">
-        <f>IF(OR(B5&gt;10000,C5&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F5" s="66" t="str">
-        <f>IF(AND(B5&gt;20000,C5&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="66" t="str" cm="1">
-        <f t="array" ref="G5">_xlfn.IFS(B5&gt;20000,"A",B5&gt;10000,"B",B5&lt;10000,"C")</f>
-        <v>B</v>
-      </c>
-      <c r="H5" s="66" t="str">
-        <f>IF(B5&gt;20000,"A",IF(B5&gt;10000,"B",IF(B5&lt;10000,"C")))</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="67" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="66">
-        <v>33641</v>
-      </c>
-      <c r="C6" s="66">
-        <v>10</v>
-      </c>
-      <c r="D6" s="66" t="str">
-        <f>IF(B6&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E6" s="66" t="str">
-        <f>IF(OR(B6&gt;10000,C6&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F6" s="66" t="str">
-        <f>IF(AND(B6&gt;20000,C6&gt;9),"30%","0")</f>
-        <v>30%</v>
-      </c>
-      <c r="G6" s="66" t="str" cm="1">
-        <f t="array" ref="G6">_xlfn.IFS(B6&gt;20000,"A",B6&gt;10000,"B",B6&lt;10000,"C")</f>
-        <v>A</v>
-      </c>
-      <c r="H6" s="66" t="str">
-        <f>IF(B6&gt;20000,"A",IF(B6&gt;10000,"B",IF(B6&lt;10000,"C")))</f>
-        <v>A</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="67" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="66">
-        <v>26146</v>
-      </c>
-      <c r="C7" s="66">
-        <v>15</v>
-      </c>
-      <c r="D7" s="66" t="str">
-        <f>IF(B7&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E7" s="66" t="str">
-        <f>IF(OR(B7&gt;10000,C7&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F7" s="66" t="str">
-        <f>IF(AND(B7&gt;20000,C7&gt;9),"30%","0")</f>
-        <v>30%</v>
-      </c>
-      <c r="G7" s="66" t="str" cm="1">
-        <f t="array" ref="G7">_xlfn.IFS(B7&gt;20000,"A",B7&gt;10000,"B",B7&lt;10000,"C")</f>
-        <v>A</v>
-      </c>
-      <c r="H7" s="66" t="str">
-        <f>IF(B7&gt;20000,"A",IF(B7&gt;10000,"B",IF(B7&lt;10000,"C")))</f>
-        <v>A</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="67" t="s">
-        <v>131</v>
-      </c>
-      <c r="B8" s="66">
-        <v>30080</v>
-      </c>
-      <c r="C8" s="66">
-        <v>4</v>
-      </c>
-      <c r="D8" s="66" t="str">
-        <f>IF(B8&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E8" s="66" t="str">
-        <f>IF(OR(B8&gt;10000,C8&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F8" s="66" t="str">
-        <f>IF(AND(B8&gt;20000,C8&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="66" t="str" cm="1">
-        <f t="array" ref="G8">_xlfn.IFS(B8&gt;20000,"A",B8&gt;10000,"B",B8&lt;10000,"C")</f>
-        <v>A</v>
-      </c>
-      <c r="H8" s="66" t="str">
-        <f>IF(B8&gt;20000,"A",IF(B8&gt;10000,"B",IF(B8&lt;10000,"C")))</f>
-        <v>A</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="67" t="s">
-        <v>130</v>
-      </c>
-      <c r="B9" s="66">
-        <v>32446</v>
-      </c>
-      <c r="C9" s="66">
-        <v>13</v>
-      </c>
-      <c r="D9" s="66" t="str">
-        <f>IF(B9&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E9" s="66" t="str">
-        <f>IF(OR(B9&gt;10000,C9&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F9" s="66" t="str">
-        <f>IF(AND(B9&gt;20000,C9&gt;9),"30%","0")</f>
-        <v>30%</v>
-      </c>
-      <c r="G9" s="66" t="str" cm="1">
-        <f t="array" ref="G9">_xlfn.IFS(B9&gt;20000,"A",B9&gt;10000,"B",B9&lt;10000,"C")</f>
-        <v>A</v>
-      </c>
-      <c r="H9" s="66" t="str">
-        <f>IF(B9&gt;20000,"A",IF(B9&gt;10000,"B",IF(B9&lt;10000,"C")))</f>
-        <v>A</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="67" t="s">
-        <v>129</v>
-      </c>
-      <c r="B10" s="66">
-        <v>13153</v>
-      </c>
-      <c r="C10" s="66">
-        <v>8</v>
-      </c>
-      <c r="D10" s="66" t="str">
-        <f>IF(B10&gt;5000,"10%","0")</f>
-        <v>10%</v>
-      </c>
-      <c r="E10" s="66" t="str">
-        <f>IF(OR(B10&gt;10000,C10&gt;4),"20%")</f>
-        <v>20%</v>
-      </c>
-      <c r="F10" s="66" t="str">
-        <f>IF(AND(B10&gt;20000,C10&gt;9),"30%","0")</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="66" t="str" cm="1">
-        <f t="array" ref="G10">_xlfn.IFS(B10&gt;20000,"A",B10&gt;10000,"B",B10&lt;10000,"C")</f>
-        <v>B</v>
-      </c>
-      <c r="H10" s="66" t="str">
-        <f>IF(B10&gt;20000,"A",IF(B10&gt;10000,"B",IF(B10&lt;10000,"C")))</f>
-        <v>B</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="65"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="65"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>